<commit_message>
Working on week 7
</commit_message>
<xml_diff>
--- a/07_1-Gas_Taxes_by_State2023.xlsx
+++ b/07_1-Gas_Taxes_by_State2023.xlsx
@@ -272,27 +272,18 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B51"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.16"/>
   </cols>
   <sheetData>
@@ -357,7 +348,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.05</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -716,12 +707,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>